<commit_message>
fix(report): restore full-bleed Letter PDF geometry via CSS @page for WeasyPrint, re-baseline golden for maintainer-updated v1.16 fixture
</commit_message>
<xml_diff>
--- a/data/input/data_ground_truth_01/descricao.xlsx
+++ b/data/input/data_ground_truth_01/descricao.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="56">
   <si>
     <t xml:space="preserve">codigo</t>
   </si>
@@ -49,6 +49,9 @@
     <t xml:space="preserve">relacao</t>
   </si>
   <si>
+    <t xml:space="preserve">categoria</t>
+  </si>
+  <si>
     <t xml:space="preserve">fontes</t>
   </si>
   <si>
@@ -64,12 +67,15 @@
     <t xml:space="preserve">Impactos para segurança alimentar</t>
   </si>
   <si>
-    <t xml:space="preserve">Consequências esperadas e resultantes das mudanças climáticas em sistemas socioecológicos relacionados à segurança alimentar.</t>
+    <t xml:space="preserve">Consequências esperadas e resultantes das mudanças climáticas em sistemas socioecológicos relacionados à segurança alimentar</t>
   </si>
   <si>
     <t xml:space="preserve">São os efeitos sobre vidas, meios de subsistência, saúde, ecossistemas, economias, sociedades, culturas, serviços e infraestrutura, devido a alterações climáticas ou eventos climáticos que se dão dentro de períodos específicos de tempo, de vulnerabilidade e de exposição da sociedade ou sistema, relacionados à segurança alimentar.&lt;br&gt;A Segurança Alimentar e Nutricional (SAN) consiste na realização do direito de todos ao acesso regular e permanente a alimentos de qualidade, em quantidade suficiente, sem comprometer o acesso a outras necessidades essenciais, tendo como base práticas alimentares promotoras de saúde, que respeitem a diversidade cultural e que sejam ambiental, cultural, econômica e socialmente sustentáveis.&lt;br&gt;&lt;br&gt;Fontes:&lt;br&gt;&lt;a href="http://www.planalto.gov.br/ccivil_03/_ato2004-2006/2006/lei/l11346.htm"&gt;BRASIL. LEI Nº 11.346, DE 15 DE SETEMBRO DE 2006. Brasília: 2006.&lt;/a&gt;&lt;br&gt;INTERGOVERNMENTAL PANEL ON CLIMATE CHANGE - IPCC. Climate Change 2014: Synthesis Report. Working Groups I, II and III to the Fifth Assessment Report of the Intergovernmental Panel on Climate Change [Core Writing Team, R.K. Pachauri and L.A. Meyer (eds.)]. IPCC, Geneva, Switzerland, 151 pp.</t>
   </si>
   <si>
+    <t xml:space="preserve">climatico</t>
+  </si>
+  <si>
     <t xml:space="preserve">AdaptaBrasil MCTI/INPE</t>
   </si>
   <si>
@@ -82,7 +88,7 @@
     <t xml:space="preserve">Índice de risco de impacto para seca</t>
   </si>
   <si>
-    <t xml:space="preserve">Risco de impacto das mudanças climáticas em sistemas socioecológicos, considerando a ameaça climática de seca.</t>
+    <t xml:space="preserve">Risco de impacto das mudanças climáticas em sistemas socioecológicos, considerando a ameaça climática de seca</t>
   </si>
   <si>
     <t xml:space="preserve">Risco de impacto das mudanças climáticas em sistemas socioecológicos, resultante da interação entre os eventos climáticos relacionados à seca, vulnerabilidade e exposição desses sistemas. Considera-se seca como um período prolongado — uma estação, um ano ou vários anos — de precipitação deficiente em comparação com a média multianual estatística para uma região que resulta em escassez de água para alguma atividade, grupo ou setor ambiental.&lt;br&gt;&lt;br&gt;Fonte:&lt;br&gt;FOOD AND AGRICULTURE ORGANIZATION/NATIONAL DROUGHT MITIGATION CENTER - FAO/NDMC.The Near East Drought Planning Manual. Food and Agriculture Organization of the United Nations (FAO): Rome: Italy, 2008.</t>
@@ -97,7 +103,7 @@
     <t xml:space="preserve">Índice de vulnerabilidade</t>
   </si>
   <si>
-    <t xml:space="preserve">Grau de suscetibilidade de um sistema socioecológico aos efeitos das mudanças climáticas, especificamente aquelas que resultam em seca.</t>
+    <t xml:space="preserve">Grau de suscetibilidade de um sistema socioecológico aos efeitos das mudanças climáticas, especificamente aquelas que resultam em seca</t>
   </si>
   <si>
     <t xml:space="preserve">Grau de suscetibilidade a danos, com potencial para mudança ou transformação do sistema socioecológico, quando confrontado com uma ameaça. A vulnerabilidade está associada às situações de sensibilidade e capacidade adaptativa do sistema socioecológico às alterações climáticas (seca). Assim, o Índice de Vulnerabilidade é resultante da composição dos índices de Sensibilidade e Capacidade Adaptativa.&lt;br&gt;&lt;br&gt;Fontes:&lt;br&gt;GALLOPÍN, G. C.. Linkages between vulnerability, resilience, and adaptive capacity. Global Environmental Change, v. 16, p. 293-303, 2006.&lt;br&gt;INTERGOVERNMENTAL PANEL ON CLIMATE CHANGE - IPCC. Climate Change 2014: Synthesis Report. Working Groups I, II and III to the Fifth Assessment Report of the Intergovernmental Panel on Climate Change [Core Writing Team, R.K. Pachauri and L.A. Meyer (eds.)]. IPCC, Geneva, Switzerland, 151 pp.</t>
@@ -109,7 +115,7 @@
     <t xml:space="preserve">Índice de exposição</t>
   </si>
   <si>
-    <t xml:space="preserve">Magnitude do contato entre o sistema socioecológico e as ameaças climáticas relacionadas à seca por meio da distribuição de elementos de superfície.</t>
+    <t xml:space="preserve">Magnitude do contato entre o sistema socioecológico e as ameaças climáticas relacionadas à seca por meio da distribuição de elementos de superfície</t>
   </si>
   <si>
     <t xml:space="preserve">Grau, duração e/ou extensão em que o sistema está sujeito à ameaça climática (seca), considerando a distribuição de elementos de superfície local (como disponibilidade hídrica, áreas degradadas, potencial agrícola, etc.), resultante da relação entre o sistema e a ameaça climática em questão. A exposição a uma ameaça particular pode ser determinada independentemente da vulnerabilidade. O Índice de Exposição é resultante da composição dos indicadores temáticos: agropecuária e fatores biofísicos, e população exposta e estrutura fundiária.&lt;br&gt;&lt;br&gt;Fontes:&lt;br&gt;ADGER, W. N.. Vulnerability. Global Environmental Change, v. 16, n. 3, p. 268-281, ago. 2006.&lt;br&gt;GALLOPÍN, G. C.. Box 1: A systemic synthesis of the relations between vulnerability, hazard, exposure and impact, aimed at policy identification. In: Economic Commission for Latin American and the Caribbean (ECLAC). Handbook for Estimating the Socio-Economic and Environmental Effects of Disasters. Mexico, D.F.: ECLAC, LC/MEX/G.S., p. 2-5, 2003.&lt;br&gt;INTERGOVERNMENTAL PANEL ON CLIMATE CHANGE - IPCC. Climate Change 2014: Synthesis Report. Working Groups I, II and III to the Fifth Assessment Report of the Intergovernmental Panel on Climate Change [Core Writing Team, R.K. Pachauri and L.A. Meyer (eds.)]. IPCC, Geneva, Switzerland, 151 pp.&lt;br&gt; KASPERSON, J. X.; KASPERSON, R. E.; TURNER II., B. L., SCHILLER, A., HSIEL, W. H.. Vulnerability to global environmental change. In: KASPERSON, J. X.; KASPERSON, R. E. (Eds.), Social Contours of Risk, vol. II. Earthscan, London, 2005. p. 245-285.</t>
@@ -124,7 +130,7 @@
     <t xml:space="preserve">Índice de ameaça climática</t>
   </si>
   <si>
-    <t xml:space="preserve">Variações climáticas relacionadas à seca, com base em um intervalo climático normal de 30 anos.</t>
+    <t xml:space="preserve">Variações climáticas relacionadas à seca, com base em um intervalo climático normal de 30 anos</t>
   </si>
   <si>
     <t xml:space="preserve">O sistema socioecológico é um dos componentes do sistema terrestre expostos às ameaças climáticas como a seca. Por convenção, o termo ameaça climática no AdaptaBrasil será utilizado para denotar fatores externos (especificamente climáticos) que interagem com o sistema socioecológico analisado e que possuem capacidade de impactar de forma significativa o sistema, seja de forma lenta ou repentina. O Índice de Ameaça Climática para a seca é resultante da composição do número de dias consecutivos secos e do Índice de Precipitação-Evapotranspiração Padronizado (do acrônimo em inglês Standardized Precipitation-Evapotranspiration Index). Devido à utilização de uma faixa de valores do AdaptaBrasil que expressam padrões de seca (valores inferiores a -0,5), os valores superiores a -0,5 foram desconsiderados e receberam NA (do inglês Not Available ou Não Disponível em tradução livre), visto que os mesmos caracterizam normalidade ou excessos de chuvas quando ponderada a precipitação. No resultado final do índice, os valores NA foram substituídos por 0 (zero), visto que isso representa a ausência de padrões de seca.&lt;br&gt;&lt;br&gt;Fontes:&lt;br&gt;GALLOPÍN, G. C.. Box 1: A systemic synthesis of the relations between vulnerability, hazard, exposure and impact, aimed at policy identification. In: Economic Commission for Latin American and the Caribbean (ECLAC). Handbook for Estimating the Socio-Economic and Environmental Effects of Disasters. Mexico, D.F.: ECLAC, LC/MEX/G.S., p. 2-5, 2003.&lt;br&gt;INTERGOVERNMENTAL PANEL ON CLIMATE CHANGE - IPCC. Climate Change 2014: Synthesis Report. Working Groups I, II and III to the Fifth Assessment Report of the Intergovernmental Panel on Climate Change [Core Writing Team, R.K. Pachauri and L.A. Meyer (eds.)]. IPCC, Geneva, Switzerland, 151 pp.</t>
@@ -139,7 +145,7 @@
     <t xml:space="preserve">Índice de sensibilidade</t>
   </si>
   <si>
-    <t xml:space="preserve">Grau em que um sistema socioecológico é potencialmente modificado ou afetado por uma ameaça climática de seca.</t>
+    <t xml:space="preserve">Grau em que um sistema socioecológico é potencialmente modificado ou afetado por uma ameaça climática de seca</t>
   </si>
   <si>
     <t xml:space="preserve">Grau em que um sistema socioecológico é potencialmente modificado ou afetado, direta ou indiretamente, adversamente ou beneficamente, por estímulos relacionados ao clima, especificamente à seca. Também pode ser entendido como a razão entre a mudança do sistema socioecológico e a unidade de quantidade de ameaça. A sensibilidade é uma propriedade inerente de um sistema socioecológico, existente antes da ameaça e independentemente da exposição desse sistema. O Índice de Sensibilidade é resultante da composição dos indicadores temáticos: produção e comercialização de alimentos, características dos produtores e dos estabelecimentos agropecuários, e saúde e consumo dos alimentos.&lt;br&gt;&lt;br&gt;Fontes:&lt;br&gt;GALLOPÍN, G. C.. Box 1: A systemic synthesis of the relations between vulnerability, hazard, exposure and impact, aimed at policy identification. In: Economic Commission for Latin American and the Caribbean (ECLAC). Handbook for Estimating the Socio-Economic and Environmental Effects of Disasters. Mexico, D.F.: ECLAC, LC/MEX/G.S., p. 2-5, 2003.&lt;br&gt;INTERGOVERNMENTAL PANEL ON CLIMATE CHANGE - IPCC. CLIMATE CHANGE 2001: impacts, adaptation and vulnerability. Contribution of Working Group II to the Third Assessment Report of the Intergovernmental Panel on Climate Change [[Core Writing Team, J. J. McCartthy; O. F. Canziani; N. A. Leary; D. J. Dokken and K. S. White (eds.)]. IPCC, Cambridge, United Kingdom, 10p.</t>
@@ -154,7 +160,7 @@
     <t xml:space="preserve">Índice de capacidade adaptativa</t>
   </si>
   <si>
-    <t xml:space="preserve">Capacidade do sistema socioecológico de se ajustar a possíveis ameaças climáticas de seca.</t>
+    <t xml:space="preserve">Capacidade do sistema socioecológico de se ajustar a possíveis ameaças climáticas de seca</t>
   </si>
   <si>
     <t xml:space="preserve">Capacidade do sistema socioecológico de se preparar e se ajustar às alterações climáticas ou aos danos climáticos potenciais relacionados à seca, principalmente para diminuir os impactos negativos, aproveitar as oportunidades ou responder às consequências. O Índice de Capacidade Adaptativa é resultante da composição dos indicadores temáticos: logística da produção e abastecimento, planejamento e gestão da segurança alimentar e nutricional, manutenção da produção agropecuária, e capacidade socioeconômica familiar.&lt;br&gt;&lt;br&gt;Fontes:&lt;br&gt;ADGER, W. N. Vulnerability. Global Environmental Change, v. 16, n. 3, p. 268–281, ago. 2006.&lt;br&gt;GALLOPÍN, G. C.. Box 1: A systemic synthesis of the relations between vulnerability, hazard, exposure and impact, aimed at policy identification. In: Economic Commission for Latin American and the Caribbean (ECLAC). Handbook for Estimating the Socio-Economic and Environmental Effects of Disasters. Mexico, D.F.: ECLAC, LC/MEX/G.S., p. 2-5, 2003.&lt;br&gt;GALLOPÍN, G. C.. Linkages between vulnerability, resilience, and adaptive capacity. Global Environmental Change, v. 16, p. 293-303, 2006.&lt;br&gt;INTERGOVERNMENTAL PANEL ON CLIMATE CHANGE - IPCC. Climate Change 2014: Synthesis Report. Working Groups I, II and III to the Fifth Assessment Report of the Intergovernmental Panel on Climate Change [Core Writing Team, R.K. Pachauri and L.A. Meyer (eds.)]. IPCC, Geneva, Switzerland, 151 pp.</t>
@@ -166,7 +172,7 @@
     <t xml:space="preserve">Produção e comercialização de alimentos</t>
   </si>
   <si>
-    <t xml:space="preserve">Capacidade do sistema socioecológico de se ajustar a possíveis ameaças climáticas de seca teste 4.</t>
+    <t xml:space="preserve">Capacidade do sistema socioecológico de se ajustar a possíveis ameaças climáticas de seca teste 4</t>
   </si>
   <si>
     <t xml:space="preserve">Sensibilidade do sistema quanto à disponibilidade de alimento e as possíveis limitações na sua comercialização no presente e no futuro considerando uma situação de seca. Essa informação é resultante da composição dos indicadores: baixa produção de alimentos básicos e não diversificação da produção local.&lt;br&gt;&lt;br&gt;Fonte:&lt;br&gt;Sistema de Informações e Análises sobre Impactos das Mudanças Climáticas – AdaptaBrasil MCTI.</t>
@@ -178,7 +184,7 @@
     <t xml:space="preserve">Características dos produtores e dos estabelecimentos agropecuários</t>
   </si>
   <si>
-    <t xml:space="preserve">Dependência dos estabelecimentos agropecuários aos aspectos que podem expressar a sensibilidade do sistema em situação de seca.</t>
+    <t xml:space="preserve">Dependência dos estabelecimentos agropecuários aos aspectos que podem expressar a sensibilidade do sistema em situação de seca</t>
   </si>
   <si>
     <t xml:space="preserve">Dependência dos estabelecimentos agropecuários aos aspectos que podem expressar a sensibilidade do sistema em situação de seca. Informação resultante da composição dos indicadores: agricultura sem práticas agrícolas sustentáveis, dependência da irrigação em grande escala, uniformidade de receitas da produção agropecuária e analfabetismo do responsável pelo estabelecimento agropecuário.&lt;br&gt;&lt;br&gt;Fonte:&lt;br&gt;Sistema de Informações e Análises sobre Impactos das Mudanças Climáticas - AdaptaBrasil MCTI.</t>
@@ -389,8 +395,11 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:L10"/>
-  <sheetFormatPr defaultColWidth="10.16015625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:M10"/>
+  <sheetFormatPr defaultColWidth="10.1640625" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="136.61"/>
+  </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -429,6 +438,9 @@
       <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
+      <c r="M1" s="1" t="s">
+        <v>12</v>
+      </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="n">
@@ -438,16 +450,16 @@
         <v>1</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="H2" s="1" t="n">
         <v>0</v>
@@ -456,10 +468,13 @@
         <v>1</v>
       </c>
       <c r="J2" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="K2" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
+      </c>
+      <c r="L2" s="1" t="s">
+        <v>19</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -470,16 +485,16 @@
         <v>2</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="G3" s="1" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="H3" s="1" t="n">
         <v>1</v>
@@ -488,12 +503,15 @@
         <v>1</v>
       </c>
       <c r="J3" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="K3" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="L3" s="1" t="n">
+        <v>18</v>
+      </c>
+      <c r="L3" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="M3" s="1" t="n">
         <v>1</v>
       </c>
     </row>
@@ -505,16 +523,16 @@
         <v>3</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="H4" s="1" t="n">
         <v>0</v>
@@ -523,12 +541,15 @@
         <v>1</v>
       </c>
       <c r="J4" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="K4" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="L4" s="1" t="n">
+        <v>18</v>
+      </c>
+      <c r="L4" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="M4" s="1" t="n">
         <v>1</v>
       </c>
     </row>
@@ -540,16 +561,16 @@
         <v>3</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="H5" s="1" t="n">
         <v>0</v>
@@ -558,12 +579,15 @@
         <v>1</v>
       </c>
       <c r="J5" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="K5" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="L5" s="1" t="n">
+        <v>18</v>
+      </c>
+      <c r="L5" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="M5" s="1" t="n">
         <v>1</v>
       </c>
     </row>
@@ -575,16 +599,16 @@
         <v>3</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="H6" s="1" t="n">
         <v>1</v>
@@ -593,12 +617,15 @@
         <v>1</v>
       </c>
       <c r="J6" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="K6" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="L6" s="1" t="n">
+        <v>18</v>
+      </c>
+      <c r="L6" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="M6" s="1" t="n">
         <v>1</v>
       </c>
     </row>
@@ -610,16 +637,16 @@
         <v>4</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="H7" s="1" t="n">
         <v>0</v>
@@ -628,12 +655,15 @@
         <v>1</v>
       </c>
       <c r="J7" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="K7" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="L7" s="1" t="n">
+        <v>18</v>
+      </c>
+      <c r="L7" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="M7" s="1" t="n">
         <v>2</v>
       </c>
     </row>
@@ -645,16 +675,16 @@
         <v>4</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="G8" s="1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="H8" s="1" t="n">
         <v>0</v>
@@ -663,12 +693,15 @@
         <v>-1</v>
       </c>
       <c r="J8" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="K8" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="L8" s="1" t="n">
+        <v>18</v>
+      </c>
+      <c r="L8" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="M8" s="1" t="n">
         <v>2</v>
       </c>
     </row>
@@ -680,16 +713,16 @@
         <v>5</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="H9" s="1" t="n">
         <v>0</v>
@@ -698,12 +731,15 @@
         <v>1</v>
       </c>
       <c r="J9" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="K9" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="L9" s="1" t="n">
+        <v>18</v>
+      </c>
+      <c r="L9" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="M9" s="1" t="n">
         <v>3</v>
       </c>
     </row>
@@ -715,16 +751,16 @@
         <v>5</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="G10" s="1" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="H10" s="1" t="n">
         <v>0</v>
@@ -733,12 +769,15 @@
         <v>1</v>
       </c>
       <c r="J10" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="K10" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="L10" s="1" t="n">
+        <v>18</v>
+      </c>
+      <c r="L10" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="M10" s="1" t="n">
         <v>3</v>
       </c>
     </row>

</xml_diff>